<commit_message>
Add requirments.text for Render Deployment
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,10 +481,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
+      <c r="A3" t="n">
+        <v>123456</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -504,6 +502,33 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>2025-12-17 11:05:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>54346`</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ted ted</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>11:12:36</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025-12-17 11:12:36</t>
         </is>
       </c>
     </row>

</xml_diff>